<commit_message>
master sheet: road rate approx Rs 5 per tonne-km (Aman)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQM6YzoCaqWWyBshTm6kGs
</commit_message>
<xml_diff>
--- a/briefs/COMPETITOR_TENDER_MASTER_2026-10-12.xlsx
+++ b/briefs/COMPETITOR_TENDER_MASTER_2026-10-12.xlsx
@@ -34265,10 +34265,12 @@
           <t>Road quote Rs per tonne-km (YOUR NUMBER)</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n"/>
+      <c r="B3" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Type your tipper rate. Leave blank to use the illustrative rate.</t>
+          <t>Aman, chat 2026-10-12: approx Rs 5 per tonne per km (approximate, not a written quote). Clear the cell to fall back to the illustrative rate.</t>
         </is>
       </c>
     </row>

</xml_diff>